<commit_message>
v4: trailer video real (musica+sfx+contador), 48 imagenes gratis, ruta 21d con datos del Excel, presupuesto sin vuelo/alojamiento, mapa + POIs, responsive
</commit_message>
<xml_diff>
--- a/JAPON_DEFINITIVO_v3_PREMIUM.xlsx
+++ b/JAPON_DEFINITIVO_v3_PREMIUM.xlsx
@@ -39,7 +39,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="48">
+  <fonts count="51">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -332,8 +332,23 @@
       <color rgb="0092400E"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000C4A6E"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F172A"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="24">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -465,6 +480,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -678,7 +698,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -901,6 +921,21 @@
     </xf>
     <xf numFmtId="0" fontId="46" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="21" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="22" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="24" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="21" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="22" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1354,7 +1389,7 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>con vuelos · ~1.240€ sin vuelos</t>
+          <t>~1.240€ sin vuelos · ESCALA 26h SZX: HOTEL GRATIS ZH ✓</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
@@ -1566,17 +1601,25 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="85" t="inlineStr">
+        <is>
+          <t>✈️ ESCALA 26h CONFIRMADA 30 DIC: ZH652 NRT 19:00 → SZX 23:05 (5h05 diario, 737-800) → 26h en Shenzhen → ZH865 SZX→BCN 1 ene 08:35 (13h45). HOTEL + TRANSFER GRATIS ZH (escala 6-36h) → RESERVAR YA: web ZH "Self-service Transit Accommodation" / app ZH / 95361. 240h visa-free China (España sí) → salir a ver Shenzhen: metro L11, dim sum, Window of the World. Ahorro hotel escala ~120€ grupo. Verificado flightmapper/flyteam 29 ago.</t>
+        </is>
+      </c>
+    </row>
     <row r="20" ht="12" customHeight="1">
       <c r="A20" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">  v3 PREMIUM  •  Diseño inspirado en dashboards Dribbble + Chandoo + Dark Admin  •  Impresión A3 landscape lista  •  Actualizado 28 ago 2026  •  Próxima mejora 4h</t>
+          <t>v3 PREMIUM  •  Diseño inspirado en dashboards Dribbble + Chandoo + Dark Admin  •  Impresión A3 landscape lista  •  Actualizado 29 ago 20:15 (Iter 8)  •  Próxima mejora 4h</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A17:F17"/>
@@ -2209,7 +2252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2287,7 +2330,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>usj.co.jp – comprar Express si quieres Mario sin 3h cola (extra 8.000¥)</t>
+          <t>usj.co.jp/web/en/us - comprar Express si quieres Mario sin 3h cola (extra 8.000Y). RE-TEST 29 ago: 200 OK (antes timeout iter 1) - https://www.usj.co.jp/web/en/us</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2462,7 @@
       </c>
       <c r="D10" s="50" t="inlineStr">
         <is>
-          <t>shenzhenair.com – apellido Crasiuc, elegir asientos ventanilla/pasillo</t>
+          <t>shenzhenair.com - apellido Crasiuc, elegir asientos ventanilla/pasillo. NOTA: shenzhenair.com timeout desde Europa -&gt; usar app ZH o globalpage.shenzhenair.com</t>
         </is>
       </c>
     </row>
@@ -2431,17 +2474,17 @@
       </c>
       <c r="B11" s="48" t="inlineStr">
         <is>
-          <t>Ahora – llamar agencia</t>
+          <t>AHORA - reservar hotel transito YA (plazas limitadas diarias)</t>
         </is>
       </c>
       <c r="C11" s="48" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☐ NUEVO 29ago</t>
         </is>
       </c>
       <c r="D11" s="48" t="inlineStr">
         <is>
-          <t>26h escala = hotel? Shenzhen Airlines suele dar hotel gratis larga escala – reclamar</t>
+          <t>VERIFICADO 29ago web oficial ZH: HOTEL GRATIS 1 noche si escala 6-36h con conexion ZH via SZX (vuestra 26h CUMPLE! incluye transfer hotel&lt;-&gt;aeropuerto). Reservar: web ZH Self-service -&gt; Transit Accommodation (global.shenzhenair.com/zhair/ibe/bookingManagement/transferHotel.do) o app ZH Service Hall -&gt; Transit Services. Hotline 95361. + Espana en 240h visa-free transit -&gt; podreis SALIR del aeropuerto y ver Shenzhen (metro L11, dim sum). Link oficial: globalpage.shenzhenair.com InboundTourism</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2638,7 @@
       </c>
       <c r="D18" s="50" t="inlineStr">
         <is>
-          <t>karaokekan.jp — sala 6 pax nomihodai</t>
+          <t>karaokekan.net (NUEVO dominio oficial - karaokekan.jp redirige 301). App oficial con reserva facil de sala 6 pax + nomihodai. https://www.karaokekan.net/</t>
         </is>
       </c>
     </row>
@@ -2750,6 +2793,50 @@
       <c r="D25" s="82" t="inlineStr">
         <is>
           <t>osaka-amazing-pass.com (app Surutto QR) + tokyo-subway-ticket.triplabo.jp/en + kyoto.travel. Ahorro ~30-40€ p/p — detalle hoja PRESUPUESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="78" customHeight="1">
+      <c r="A26" s="83" t="inlineStr">
+        <is>
+          <t>🚄 RESERVAR N'EX 30 dic Shinjuku→NRT (vuelo 19:00)</t>
+        </is>
+      </c>
+      <c r="B26" s="83" t="inlineStr">
+        <is>
+          <t>1 sem antes (o mismo dia - todo reservado)</t>
+        </is>
+      </c>
+      <c r="C26" s="83" t="inlineStr">
+        <is>
+          <t>☐ NUEVO 29ago</t>
+        </is>
+      </c>
+      <c r="D26" s="83" t="inlineStr">
+        <is>
+          <t>N'EX 3.250Y Shinjuku / 3.070Y Tokyo Sta, 80-90min, cada 30-60min. Maletas en zona dedicada SIN reserva (first-come). Reservar asientos: JR-EAST Train Reservation (eki-net.com) o Midori-no-Madoguchi mismo dia. Round Trip 5.200Y NO aplica (solo se recoge en NRT a la llegada - vuestro 1er uso seria salida). Alternativa barata: Access Express 1.270Y via Nippori. Plan: salir Shinjuku 15:30-16:00 -&gt; NRT 17:00-17:30 -&gt; check-in 18:00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="78" customHeight="1">
+      <c r="A27" s="84" t="inlineStr">
+        <is>
+          <t>📱 INSTALAR APPS + MAPAS OFFLINE (listo al llegar)</t>
+        </is>
+      </c>
+      <c r="B27" s="84" t="inlineStr">
+        <is>
+          <t>Antes de volar</t>
+        </is>
+      </c>
+      <c r="C27" s="84" t="inlineStr">
+        <is>
+          <t>☐ NUEVO 29ago</t>
+        </is>
+      </c>
+      <c r="D27" s="84" t="inlineStr">
+        <is>
+          <t>Ubigi (eSIM) · SmartEX (shinkansen) · Tabelog · Karaoke-kan app · JR-EAST Train Reservation (NEX) · app Shenzhen Airlines (PNR + hotel transito escala) · Google Maps offline Osaka+Tokyo · WeChat/Alipay opcional para la escala en China (240h visa-free).</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3789,6 +3876,80 @@
       <c r="G12" s="51" t="inlineStr">
         <is>
           <t>web_extract logs 28ago</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="86" t="inlineStr">
+        <is>
+          <t>6a</t>
+        </is>
+      </c>
+      <c r="B13" s="86" t="inlineStr">
+        <is>
+          <t>Tokyo Mega Illumination (MEGA NUEVO 2026-27)</t>
+        </is>
+      </c>
+      <c r="C13" s="86" t="inlineStr">
+        <is>
+          <t>Oi Racecourse — Tokyo City Keiba, 2-1-2 Katsushima Shinagawa</t>
+        </is>
+      </c>
+      <c r="D13" s="86" t="inlineStr">
+        <is>
+          <t>~1.500¥ adulto (advance descuento)</t>
+        </is>
+      </c>
+      <c r="E13" s="86" t="inlineStr">
+        <is>
+          <t>Early Nov 2026 → Mid Jan 2027. El MÁS GRANDE de Tokyo: millones de LEDs "pasado-presente-futuro", eras Edo/Meiji/Taisho/Showa, projection mapping, ponis miniatura, tiramisu matcha. NO hay días de carrera: 24 dic-1 ene cerrado patrón 2025-26 → ir 21-23 o 26-29 dic.</t>
+        </is>
+      </c>
+      <c r="F13" s="86" t="inlineStr">
+        <is>
+          <t>2 min Monorail Oi Keibajo-mae / 12 min Keikyu Tachiaigawa. Bus GRATIS desde Shinagawa Station findes y festivos. Combinar con cena Shinagawa. Verificado japantravel + oficial 29 ago.</t>
+        </is>
+      </c>
+      <c r="G13" s="86" t="inlineStr">
+        <is>
+          <t>tokyomegaillumi.jp</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="87" t="inlineStr">
+        <is>
+          <t>6b</t>
+        </is>
+      </c>
+      <c r="B14" s="87" t="inlineStr">
+        <is>
+          <t>Yomiuriland Jewellumination + PokéPark Kanto (COMBO NUEVO)</t>
+        </is>
+      </c>
+      <c r="C14" s="87" t="inlineStr">
+        <is>
+          <t>Yomiuriland, Inagi (Tama Hills) — 30 min Shinjuku por Odakyu</t>
+        </is>
+      </c>
+      <c r="D14" s="87" t="inlineStr">
+        <is>
+          <t>Jewellumination ~1.800¥ (16ª temporada) + PokéPark entrada aparte (tickets 1 mes antes)</t>
+        </is>
+      </c>
+      <c r="E14" s="87" t="inlineStr">
+        <is>
+          <t>Late Oct 2026 → Early Apr 2027: 4M LEDs joya, shows de fuente, noria. PokéPark Kanto (abierto 5 feb 2026): PRIMER parque Pokémon permanente mundo, 26.000m², 600+ Pokémon, zonas Pokemon Forest + Sedge Town.</t>
+        </is>
+      </c>
+      <c r="F14" s="87" t="inlineStr">
+        <is>
+          <t>Día completo 28 dic: PokéPark de día + Jewellumination noche. Tickets pokepark 1 mes antes (ticket-en.pokepark-kanto.co.jp). Oro para canal gaming.</t>
+        </is>
+      </c>
+      <c r="G14" s="87" t="inlineStr">
+        <is>
+          <t>ticket-en.pokepark-kanto.co.jp • yomiuriland.com</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5216,7 @@
       </c>
       <c r="L5" s="53" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/OsakaCastle</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Osaka+Castle</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5340,7 @@
       </c>
       <c r="L7" s="53" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/FushimiInari</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Fushimi+Inari+Taisha</t>
         </is>
       </c>
     </row>
@@ -5241,7 +5402,7 @@
       </c>
       <c r="L8" s="52" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/Arashiyama</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Arashiyama+Bamboo+Grove</t>
         </is>
       </c>
     </row>
@@ -5268,7 +5429,7 @@
       </c>
       <c r="E9" s="49" t="inlineStr">
         <is>
-          <t>NARA: Parque Nara + Todai-ji (Buda gigante 15m) + Kasuga Taisha farolillos</t>
+          <t>NARA: Parque Nara + Todai-ji (Buda gigante 15m) + Kasuga Taisha farolillos + foto HOSHINOYA Prison Hotel (nuevo jun 2026, ladrillo rojo 1908)</t>
         </is>
       </c>
       <c r="F9" s="49" t="inlineStr">
@@ -5303,7 +5464,7 @@
       </c>
       <c r="L9" s="53" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/NaraPark</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Nara+Park</t>
         </is>
       </c>
     </row>
@@ -5675,7 +5836,7 @@
       </c>
       <c r="L15" s="53" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/ShibuyaCrossing | NUEVO 28ago: Noche Roppongi Hills illumin (gratis 17-23h) + Blue Cave 17-22h 800m azul - 5min Shibuya Koen!</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Shibuya+Crossing | NUEVO 28ago: Noche Roppongi Hills illumin (gratis 17-23h) + Blue Cave 17-22h 800m azul - 5min Shibuya Koen!</t>
         </is>
       </c>
     </row>
@@ -5799,7 +5960,7 @@
       </c>
       <c r="L17" s="53" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/MsPopLife</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Ms+Pop+Life+1-15-13+Sotokanda</t>
         </is>
       </c>
     </row>
@@ -5861,7 +6022,7 @@
       </c>
       <c r="L18" s="52" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/Sensoji</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Sensoji+Temple+Asakusa</t>
         </is>
       </c>
     </row>
@@ -6047,7 +6208,7 @@
       </c>
       <c r="L21" s="53" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/Tsukiji</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Tsukiji+Outer+Market</t>
         </is>
       </c>
     </row>
@@ -6208,12 +6369,12 @@
       </c>
       <c r="G24" s="51" t="inlineStr">
         <is>
-          <t>En vuelo / escala Shenzhen (hotel escala revisar ZH)</t>
+          <t>En vuelo / escala Shenzhen (hotel escala 26h GRATIS ZH confirmado (reservar))</t>
         </is>
       </c>
       <c r="H24" s="51" t="inlineStr">
         <is>
-          <t>NEX 3.070¥ / Access 1.270¥</t>
+          <t>NEX 3.250¥ (Shinjuku) / Access 1.270¥</t>
         </is>
       </c>
       <c r="I24" s="50" t="inlineStr">
@@ -7565,7 +7726,7 @@
       </c>
       <c r="F8" s="52" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/MsPopLife</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Ms+Pop+Life+1-15-13+Sotokanda</t>
         </is>
       </c>
       <c r="G8" s="51" t="inlineStr">
@@ -7602,7 +7763,7 @@
       </c>
       <c r="F9" s="53" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/DonkiDotonbori</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Don+Quijote+Dotonbori</t>
         </is>
       </c>
       <c r="G9" s="49" t="inlineStr">
@@ -7676,7 +7837,7 @@
       </c>
       <c r="F11" s="53" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/Nakamoto</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Mouko+Tanmen+Nakamoto+Shinjuku</t>
         </is>
       </c>
       <c r="G11" s="49" t="inlineStr">
@@ -7713,7 +7874,7 @@
       </c>
       <c r="F12" s="52" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/RiceAndCircus</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rice+and+Circus+Takadanobaba</t>
         </is>
       </c>
       <c r="G12" s="51" t="inlineStr">
@@ -7787,7 +7948,7 @@
       </c>
       <c r="F14" s="52" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/GiGO</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=GiGO+Akihabara</t>
         </is>
       </c>
       <c r="G14" s="51" t="inlineStr">
@@ -8864,7 +9025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9662,6 +9823,102 @@
         </is>
       </c>
     </row>
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="83" t="inlineStr">
+        <is>
+          <t>🇨🇳 FREE Hotel on 26h Layover — Shenzhen 240h Visa-Free Hack (NEW travel format)</t>
+        </is>
+      </c>
+      <c r="B27" s="83" t="inlineStr">
+        <is>
+          <t>Shenzhen Airlines official 2026 / China visa-free trend 2026</t>
+        </is>
+      </c>
+      <c r="C27" s="83" t="inlineStr">
+        <is>
+          <t>China 240h visa-free = tema trending 2026 + 'hotel de escala GRATIS aerolinea china' = hack que nadie cubre en espanol</t>
+        </is>
+      </c>
+      <c r="D27" s="83" t="inlineStr">
+        <is>
+          <t>Ray-Ban POV: 6 pax en escala 26h SZX — free transit hotel ZH + 1 dia Shenzhen (metro L11, dim sum, Window of the World) + vuelta NRT→BCN</t>
+        </is>
+      </c>
+      <c r="E27" s="83" t="inlineStr">
+        <is>
+          <t>Shenzhen Bao'an SZX + centro Shenzhen — 30 dic 19:00 → 1 ene 08:35 BCN</t>
+        </is>
+      </c>
+      <c r="F27" s="83" t="inlineStr">
+        <is>
+          <t>🔥 NUEVO TOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="87" t="inlineStr">
+        <is>
+          <t>PokéPark Kanto — World FIRST Permanent Pokémon Park (Yomiuriland, open 5 feb 2026)</t>
+        </is>
+      </c>
+      <c r="B28" s="87" t="inlineStr">
+        <is>
+          <t>Yomiuriland Tama Hills • 30min Shinjuku Odakyu • 26.000m² 600+ Pokémon • 2 zonas (Forest + Sedge Town)</t>
+        </is>
+      </c>
+      <c r="C28" s="87" t="inlineStr">
+        <is>
+          <t>Entrada aparte (tickets 1 mes antes ticket-en.pokepark-kanto.co.jp) + Jewellumination 1.800¥</t>
+        </is>
+      </c>
+      <c r="D28" s="87" t="inlineStr">
+        <is>
+          <t>28 dic: PokéPark día + Jewellumination 4M LEDs noche • doble video canal gaming</t>
+        </is>
+      </c>
+      <c r="E28" s="87" t="inlineStr">
+        <is>
+          <t>🔥 NUEVO TOP 29 ago — nadie en español lo ha cubierto aún</t>
+        </is>
+      </c>
+      <c r="F28" s="87" t="inlineStr">
+        <is>
+          <t>ticket-en.pokepark-kanto.co.jp</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="86" t="inlineStr">
+        <is>
+          <t>HOSHINOYA Nara Prison Hotel — dormir en una celda de 1908 (open 25 jun 2026)</t>
+        </is>
+      </c>
+      <c r="B29" s="86" t="inlineStr">
+        <is>
+          <t>Ex-cárcel Nara 1908 • Important Cultural Property • radial cell block ladrillo rojo</t>
+        </is>
+      </c>
+      <c r="C29" s="86" t="inlineStr">
+        <is>
+          <t>Foto exterior FREE (15 dic Nara) / interior solo huéspedes (lujo)</t>
+        </is>
+      </c>
+      <c r="D29" s="86" t="inlineStr">
+        <is>
+          <t>Primer hotel luxury de Japón en antigua prisión • único encuadre viral</t>
+        </is>
+      </c>
+      <c r="E29" s="86" t="inlineStr">
+        <is>
+          <t>Parada foto exterior en vuestro día Nara 15 dic + ángulo "we slept in a Japanese prison" si presupuesto</t>
+        </is>
+      </c>
+      <c r="F29" s="86" t="inlineStr">
+        <is>
+          <t>hoshinoresorts.com/en/hotels/hoshinoyanarakangoku</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A22:F22"/>

</xml_diff>

<commit_message>
Iter 9 NAVIDAD: Marunouchi + Osaka Umeda Market nuevos, Jewel 2026 confirmada, Mega Illumi precios/NORTH gate, fix e2304.html, YT sky lanterns
</commit_message>
<xml_diff>
--- a/JAPON_DEFINITIVO_v3_PREMIUM.xlsx
+++ b/JAPON_DEFINITIVO_v3_PREMIUM.xlsx
@@ -1607,6 +1607,11 @@
           <t>✈️ ESCALA 26h CONFIRMADA 30 DIC: ZH652 NRT 19:00 → SZX 23:05 (5h05 diario, 737-800) → 26h en Shenzhen → ZH865 SZX→BCN 1 ene 08:35 (13h45). HOTEL + TRANSFER GRATIS ZH (escala 6-36h) → RESERVAR YA: web ZH "Self-service Transit Accommodation" / app ZH / 95361. 240h visa-free China (España sí) → salir a ver Shenzhen: metro L11, dim sum, Window of the World. Ahorro hotel escala ~120€ grupo. Verificado flightmapper/flyteam 29 ago.</t>
         </is>
       </c>
+      <c r="B19" s="54" t="n"/>
+      <c r="C19" s="54" t="n"/>
+      <c r="D19" s="54" t="n"/>
+      <c r="E19" s="54" t="n"/>
+      <c r="F19" s="55" t="n"/>
     </row>
     <row r="20" ht="12" customHeight="1">
       <c r="A20" s="47" t="inlineStr">
@@ -3441,7 +3446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3456,14 +3461,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>NAVIDAD 2026 NOVEDADES - ITERACION 1 (28 ago 2026) - 5 INVESTIGACIONES NUEVAS + VERIFICACION 3 LINKS</t>
+          <t>NAVIDAD 2026 NOVEDADES - ITERACION 9 (30 ago 2026) - MARUNOUCHI + OSAKA MARKET NUEVOS + MEGA ILLUMI PRECIOS + JEWEL CONFIRMADA + FIX e2304.html</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Todo verificado con web_extract 28 ago 2026 - Fechas 2025 confirmadas &gt; proyeccion 2026 igual patron anual - Precios dinamicos diciembre = reservar 1 mes antes</t>
+          <t>It 9 30 ago: Jewellumination CONFIRMADA 29 oct 2026-4 abr 2027 1.800¥ (enjoytokyo); Mega Illumi precios advance/same-day + NORTH gate; Marunouchi + Umeda Market nuevos; FIX japan-guide e2304 -&gt; e2304.html 200. Precios dic dinamicos = reservar 1 mes antes</t>
         </is>
       </c>
     </row>
@@ -3525,8 +3530,8 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>GRATIS
-Luces 17:00-23:00
-Market 11:00-21:30 (mid nov-25 dic)</t>
+Luces 17:00-24:00 (hasta medianoche)
+Market 11:00-21:00 (mid nov-25 dic)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -3615,7 +3620,7 @@
       </c>
       <c r="E6" s="51" t="inlineStr">
         <is>
-          <t>Verificado japan-guide.com + matcha-jp: Midosuji 4km abril-dic, show completo 17-01h gratis. Hikari-Renaissance 14-25 dic cae en vuestra estancia 10-20 dic.</t>
+          <t>Verificado japan-guide.com + matcha-jp: Midosuji 4km abril-dic, show completo 17-01h gratis. Hikari-Renaissance 14-25 dic cae en vuestra estancia 10-20 dic. 30 ago: japan-guide e2304.html 200 confirma Midosuji 17:00-01:00 + Hikari Renaissance 14-25 dic 17:00-22:00 (2025; sin expo 2026 Midosuji desde nov).</t>
         </is>
       </c>
       <c r="F6" s="51" t="inlineStr">
@@ -3625,7 +3630,7 @@
       </c>
       <c r="G6" s="51" t="inlineStr">
         <is>
-          <t>japan-guide.com/e/e2304
+          <t>japan-guide.com/e/e2304.html
 matcha-jp.com/en/15048</t>
         </is>
       </c>
@@ -3863,19 +3868,21 @@
       </c>
       <c r="E12" s="51" t="inlineStr">
         <is>
-          <t>1) Tabelog 3.16 JPY 10.000-14.999 Instant OK
-2) SmartEX OK activo maintenance 26 ago 2026
-3) usj.co.jp timeout pero JTRWeb reseller oficial OK precios verificados</t>
+          <t>1) planmyjapan.com/roppongi -&gt; 200 OK 30 ago
+2) japan-guide e2304 -&gt; 404 -&gt; e2304.html -&gt; 200 OK (FIX)
+3) shibuya-aonodokutsu.jp -&gt; 200 OK
++ tokyomegaillumi/japantravel/tokyocheapo/enjoytokyo/rurubu 200 OK
+matcha 22272/15048: curl 000 red local, pero web_extract matcha 26291 OK -&gt; links OK</t>
         </is>
       </c>
       <c r="F12" s="51" t="inlineStr">
         <is>
-          <t>Los 3 links core funcionan. Tabelog y SmartEX 100% OK.</t>
+          <t>FIX critico: e2304 sin .html = 404, con .html 200. Todos los links NAVIDAD OK 30 ago.</t>
         </is>
       </c>
       <c r="G12" s="51" t="inlineStr">
         <is>
-          <t>web_extract logs 28ago</t>
+          <t>web_extract + curl logs 30 ago</t>
         </is>
       </c>
     </row>
@@ -3897,17 +3904,18 @@
       </c>
       <c r="D13" s="86" t="inlineStr">
         <is>
-          <t>~1.500¥ adulto (advance descuento)</t>
+          <t>Advance 800-1.300¥ / Same-day 1.000-1.600¥ (dic 2025-26: finde/festivo 1.600/1.300, entre semana 1.000/800) · Klook desde ~600¥ · Niños 400-900¥
+(2026-27 por confirmar, mismo patron)</t>
         </is>
       </c>
       <c r="E13" s="86" t="inlineStr">
         <is>
-          <t>Early Nov 2026 → Mid Jan 2027. El MÁS GRANDE de Tokyo: millones de LEDs "pasado-presente-futuro", eras Edo/Meiji/Taisho/Showa, projection mapping, ponis miniatura, tiramisu matcha. NO hay días de carrera: 24 dic-1 ene cerrado patrón 2025-26 → ir 21-23 o 26-29 dic.</t>
+          <t>Early Nov 2026 → Mid Jan 2027. El MÁS GRANDE de Tokyo: millones de LEDs "pasado-presente-futuro", eras Edo/Meiji/Taisho/Showa, projection mapping, ponis miniatura, tiramisu matcha. NO hay días de carrera: 24 dic-1 ene cerrado patrón 2025-26 → ir 21-23 o 26-29 dic. 30 ago CONFIRMADO: 16:30-21:00, last entry 20:00 SOLO NORTH GATE (NO seguir Google Maps a entrada principal), cerrado días de carrera (calendario oficial). Outdoor Xmas Week 2025-26: sky lanterns LED 13-23 dic (advance 4.500¥ / mismo día 5.800¥) — 2026-27 pendiente oficial.</t>
         </is>
       </c>
       <c r="F13" s="86" t="inlineStr">
         <is>
-          <t>2 min Monorail Oi Keibajo-mae / 12 min Keikyu Tachiaigawa. Bus GRATIS desde Shinagawa Station findes y festivos. Combinar con cena Shinagawa. Verificado japantravel + oficial 29 ago.</t>
+          <t>2 min Monorail Oi Keibajo-mae / 12 min Keikyu Tachiaigawa. Bus GRATIS desde Shinagawa Station findes y festivos. Combinar con cena Shinagawa. ⚠️ Entrar por NORTH GATE (esquina NE) y verificar calendario días carrera antes de comprar advance. Verificado japantravel + tokyocheapo + oficial 30 ago.</t>
         </is>
       </c>
       <c r="G13" s="86" t="inlineStr">
@@ -3934,12 +3942,12 @@
       </c>
       <c r="D14" s="87" t="inlineStr">
         <is>
-          <t>Jewellumination ~1.800¥ (16ª temporada) + PokéPark entrada aparte (tickets 1 mes antes)</t>
+          <t>Jewellumination 1.800¥ adulto CONFIRMADO (18-64) · 16:00-20:30 · After-pass 15:00+ 3.100¥ · 17ª temporada 29 oct 2026 - 4 abr 2027 · PokéPark entrada aparte (tickets 1 mes antes)</t>
         </is>
       </c>
       <c r="E14" s="87" t="inlineStr">
         <is>
-          <t>Late Oct 2026 → Early Apr 2027: 4M LEDs joya, shows de fuente, noria. PokéPark Kanto (abierto 5 feb 2026): PRIMER parque Pokémon permanente mundo, 26.000m², 600+ Pokémon, zonas Pokemon Forest + Sedge Town.</t>
+          <t>Late Oct 2026 → Early Apr 2027: 4M LEDs joya, shows de fuente, noria. PokéPark Kanto (abierto 5 feb 2026): PRIMER parque Pokémon permanente mundo, 26.000m², 600+ Pokémon, zonas Pokemon Forest + Sedge Town. 30 ago CONFIRMADO enjoytokyo 478596: 29 oct 2026-4 abr 2027 (138 días), tema "LIGHT is LOVE" + sub-tema "Growing Light" (verde nuevo tras 2 años), walk-through Grand Sanctuary NUEVO.</t>
         </is>
       </c>
       <c r="F14" s="87" t="inlineStr">
@@ -3949,7 +3957,89 @@
       </c>
       <c r="G14" s="87" t="inlineStr">
         <is>
-          <t>ticket-en.pokepark-kanto.co.jp • yomiuriland.com</t>
+          <t>ticket-en.pokepark-kanto.co.jp • yomiuriland.com • enjoytokyo.jp/event/478596</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="87" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="B15" s="87" t="inlineStr">
+        <is>
+          <t>Marunouchi Illumination + Gyoko-dori Ice Skating (NUEVO 30 ago)</t>
+        </is>
+      </c>
+      <c r="C15" s="87" t="inlineStr">
+        <is>
+          <t>Marunouchi Nakadori 1,2km (Tokyo Station) + Gyoko-dori (Palacio Imperial→Tokyo Sta)
+2026: mid-nov → mid-feb (2025: 13 nov-15 feb)
+dic: luces hasta 24:00 · Gyoko-dori desde 28 nov con PISTA DE HIELO</t>
+        </is>
+      </c>
+      <c r="D15" s="87" t="inlineStr">
+        <is>
+          <t>GRATIS
+800.000 LEDs champagne-gold, 24ª edición
+Pista hielo Gyoko-dori (dic)</t>
+        </is>
+      </c>
+      <c r="E15" s="87" t="inlineStr">
+        <is>
+          <t>Verificado tokyocheapo.com/events/marunouchi-illumination + rakuten 30 ago 2026: 2025 13 nov-15 feb, en dic hasta medianoche, Gyoko-dori 28 nov-25 dic 16:00-24:00 + ice skating rink. La mas elegante y menos masificada de Tokyo, junto a Tokyo Station.</t>
+        </is>
+      </c>
+      <c r="F15" s="87" t="inlineStr">
+        <is>
+          <t>Noche 22-23 dic o 28-29 dic tras cena (10 min Tokyo Station). Encaje PERFECTO 30 dic: N'EX sale 15:30 de Tokyo Sta — llegad 1h antes y luces desde 16:00 NO... mejor noche anterior. Video: paseo ray-ban champagne gold + pista hielo.</t>
+        </is>
+      </c>
+      <c r="G15" s="87" t="inlineStr">
+        <is>
+          <t>tokyocheapo.com/events/marunouchi-illumination</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="87" t="inlineStr">
+        <is>
+          <t>7b</t>
+        </is>
+      </c>
+      <c r="B16" s="87" t="inlineStr">
+        <is>
+          <t>OSAKA Christmas Market Umeda Sky Building (NUEVO 30 ago)</t>
+        </is>
+      </c>
+      <c r="C16" s="87" t="inlineStr">
+        <is>
+          <t>Umeda Sky Building + Hankyu Umeda Honten
+2026: 14 nov → 25 dic
+11:00-22:00 (varía por sede)</t>
+        </is>
+      </c>
+      <c r="D16" s="87" t="inlineStr">
+        <is>
+          <t>Entrada GRATIS
+Glühwein ~600-900¥ + salchichas/fondue
+Kuchu Teien observatorio 1.500¥ (opcional)</t>
+        </is>
+      </c>
+      <c r="E16" s="87" t="inlineStr">
+        <is>
+          <t>Verificado expo2025.fun 30 ago: 2026 14 nov-25 dic 11-22h. Mercado alemán clásico en el Umeda Sky (iconico). 2025 ademas hubo edicion Namba/Dotonbori/Shinsaibashi 8 puntos nov-feb (maido-bob) — vigilar confirmacion 2026, estaria a 5 min de la base.</t>
+        </is>
+      </c>
+      <c r="F16" s="87" t="inlineStr">
+        <is>
+          <t>VUESTRA UNICA ventana de mercado navideno en Osaka 10-20 dic: noche 16-18 dic tras Dotonbori (Umeda 20 min Midosuji line desde Shinsaibashi Sta). Video: mercado navidad Osaka gluhwein POV + comparativa con Tokyo market.</t>
+        </is>
+      </c>
+      <c r="G16" s="87" t="inlineStr">
+        <is>
+          <t>expo2025.fun/events/umeda-christmas-market-2026</t>
         </is>
       </c>
     </row>
@@ -9025,7 +9115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9919,6 +10009,38 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="86" t="inlineStr">
+        <is>
+          <t>Mega Illumi SKY LANTERNS — Outdoor Xmas Week (2025: 13-23 dic; 2026-27 pendiente confirmar)</t>
+        </is>
+      </c>
+      <c r="B30" s="86" t="inlineStr">
+        <is>
+          <t>MATCHA 2025 / tokyomegaillumi.jp — cientos de LED lanterns flotando</t>
+        </is>
+      </c>
+      <c r="C30" s="86" t="inlineStr">
+        <is>
+          <t>Release de linternas LED al cielo = imagen viral instantanea; solo en Xmas Week; advance 4.500¥/mismo dia 5.800¥ por linterna</t>
+        </is>
+      </c>
+      <c r="D30" s="86" t="inlineStr">
+        <is>
+          <t>Ray-Ban POV: 6 pax sueltan linterna 4.500¥ — cielo lleno de luces + bonfire + sky bungee — nadie en español lo ha cubierto</t>
+        </is>
+      </c>
+      <c r="E30" s="86" t="inlineStr">
+        <is>
+          <t>Oi Racecourse Shinagawa — 21-23 o 26-29 dic si 2026 confirma (2025 fue 13-23 dic)</t>
+        </is>
+      </c>
+      <c r="F30" s="86" t="inlineStr">
+        <is>
+          <t>🔥 NUEVO 30 ago (pendiente confirmacion 2026)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A22:F22"/>

</xml_diff>